<commit_message>
feat: add technical document fields to product schema and update bulk import utilities
</commit_message>
<xml_diff>
--- a/public/importer_template.xlsx
+++ b/public/importer_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:O3"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="45.83203125" customWidth="1"/>
@@ -411,6 +411,9 @@
     <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
     <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="35.83203125" customWidth="1"/>
+    <col min="14" max="14" width="35.83203125" customWidth="1"/>
+    <col min="15" max="15" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,6 +453,15 @@
       <c r="L1" t="str">
         <v>BIM Revit File</v>
       </c>
+      <c r="M1" t="str">
+        <v>Technical Document - Control Gear</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Technical Document - Containing Product</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Technical Document - Light Source</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -488,6 +500,15 @@
       <c r="L2" t="str">
         <v>triona_round.rfa</v>
       </c>
+      <c r="M2" t="str">
+        <v>triona_control_gear.pdf</v>
+      </c>
+      <c r="N2" t="str">
+        <v>triona_containing_product.pdf</v>
+      </c>
+      <c r="O2" t="str">
+        <v>triona_light_source.pdf</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -526,10 +547,19 @@
       <c r="L3" t="str">
         <v>triona_round.rfa</v>
       </c>
+      <c r="M3" t="str">
+        <v>triona_control_gear.pdf</v>
+      </c>
+      <c r="N3" t="str">
+        <v>triona_containing_product.pdf</v>
+      </c>
+      <c r="O3" t="str">
+        <v>triona_light_source.pdf</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>